<commit_message>
-added imerg_30min.xslx -changed domain of tcwv_wind_anomaly.py
</commit_message>
<xml_diff>
--- a/imerg_3hr.xlsx
+++ b/imerg_3hr.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Damius\Documents\Palawan_Shear_Line\Palawan_Shear_Line\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DJEV\Documents\Palawan_Shear_Line\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426BBAB4-AB69-4B08-AC9A-546DB31E5853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A62E470-408C-4DEA-B509-9F15625D4818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{A1EB678B-CB49-46E6-BA70-D9F7025CB109}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{A1EB678B-CB49-46E6-BA70-D9F7025CB109}"/>
   </bookViews>
   <sheets>
     <sheet name="imerg_3hr" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>Time</t>
   </si>
@@ -76,6 +77,66 @@
   </si>
   <si>
     <t>OBS</t>
+  </si>
+  <si>
+    <t>09_01</t>
+  </si>
+  <si>
+    <t>09_02</t>
+  </si>
+  <si>
+    <t>09_03</t>
+  </si>
+  <si>
+    <t>09_04</t>
+  </si>
+  <si>
+    <t>09_05</t>
+  </si>
+  <si>
+    <t>09_07</t>
+  </si>
+  <si>
+    <t>09_08</t>
+  </si>
+  <si>
+    <t>09_09</t>
+  </si>
+  <si>
+    <t>09_10</t>
+  </si>
+  <si>
+    <t>09_11</t>
+  </si>
+  <si>
+    <t>09_13</t>
+  </si>
+  <si>
+    <t>09_14</t>
+  </si>
+  <si>
+    <t>09_15</t>
+  </si>
+  <si>
+    <t>09_16</t>
+  </si>
+  <si>
+    <t>09_17</t>
+  </si>
+  <si>
+    <t>09_19</t>
+  </si>
+  <si>
+    <t>09_20</t>
+  </si>
+  <si>
+    <t>09_21</t>
+  </si>
+  <si>
+    <t>09_22</t>
+  </si>
+  <si>
+    <t>09_23</t>
   </si>
 </sst>
 </file>
@@ -2192,12 +2253,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{486EE33A-36C3-493C-ABC8-35286F860A06}">
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2208,7 +2269,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>3.34</v>
       </c>
@@ -2216,7 +2277,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2227,7 +2288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>0.26</v>
       </c>
@@ -2235,7 +2296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2246,7 +2307,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>0</v>
       </c>
@@ -2254,7 +2315,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -2265,7 +2326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>19.739999999999998</v>
       </c>
@@ -2273,7 +2334,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2284,7 +2345,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>90.56</v>
       </c>
@@ -2292,7 +2353,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -2303,7 +2364,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>32.33</v>
       </c>
@@ -2311,7 +2372,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -2322,7 +2383,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>6.18</v>
       </c>
@@ -2330,7 +2391,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -2341,7 +2402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>17.46</v>
       </c>
@@ -2349,7 +2410,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -2360,7 +2421,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>103.33</v>
       </c>
@@ -2368,7 +2429,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -2379,7 +2440,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>39.159999999999997</v>
       </c>
@@ -2387,7 +2448,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -2398,7 +2459,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>42.41</v>
       </c>
@@ -2406,7 +2467,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -2417,7 +2478,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>50.63</v>
       </c>
@@ -2425,7 +2486,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -2436,7 +2497,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f>SUM(B2:B25)</f>
         <v>916.7399999999999</v>
@@ -2451,4 +2512,376 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1855A55-AE8C-4B24-8657-B032129A7CD0}">
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>8.5</v>
+      </c>
+      <c r="C2">
+        <v>7.7</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>15.5</v>
+      </c>
+      <c r="C3">
+        <v>1.7</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>3.1</v>
+      </c>
+      <c r="C5">
+        <v>0.1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>0.2</v>
+      </c>
+      <c r="C7">
+        <v>0.7</v>
+      </c>
+      <c r="D7">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>0.5</v>
+      </c>
+      <c r="C8">
+        <v>0.2</v>
+      </c>
+      <c r="D8">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10">
+        <v>0.6</v>
+      </c>
+      <c r="C10">
+        <v>1.4</v>
+      </c>
+      <c r="D10">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11">
+        <v>1.3</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>0.1</v>
+      </c>
+      <c r="C12">
+        <v>0.5</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14">
+        <v>0.7</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19">
+        <v>0.2</v>
+      </c>
+      <c r="C19">
+        <v>0.1</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0.1</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22">
+        <v>0.3</v>
+      </c>
+      <c r="C22">
+        <v>4.5</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23">
+        <v>0.6</v>
+      </c>
+      <c r="C23">
+        <v>1.7</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24">
+        <v>0.1</v>
+      </c>
+      <c r="C24">
+        <v>0.3</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25">
+        <v>0.1</v>
+      </c>
+      <c r="C25">
+        <v>0.9</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>